<commit_message>
Motor exposure fix ((end-start+1)/365) + CV rerun (deviance 12,029 to 107.8) + motor v002 + combined v006 + AI log
</commit_message>
<xml_diff>
--- a/Excel files/motor_tweedie_xgb_results.xlsx
+++ b/Excel files/motor_tweedie_xgb_results.xlsx
@@ -473,10 +473,10 @@
         <v>198354</v>
       </c>
       <c r="D2" t="n">
-        <v>16135.84157143364</v>
+        <v>111.9864789645709</v>
       </c>
       <c r="E2" t="n">
-        <v>266.333740234375</v>
+        <v>237.0145111083984</v>
       </c>
       <c r="F2" t="n">
         <v>337.4496127630399</v>
@@ -493,10 +493,10 @@
         <v>198354</v>
       </c>
       <c r="D3" t="n">
-        <v>13035.29982087767</v>
+        <v>106.4365399878114</v>
       </c>
       <c r="E3" t="n">
-        <v>264.808349609375</v>
+        <v>237.4583282470703</v>
       </c>
       <c r="F3" t="n">
         <v>327.1612462566926</v>
@@ -513,10 +513,10 @@
         <v>198353</v>
       </c>
       <c r="D4" t="n">
-        <v>3510.598620545675</v>
+        <v>104.6877436476355</v>
       </c>
       <c r="E4" t="n">
-        <v>263.4286804199219</v>
+        <v>239.5449676513672</v>
       </c>
       <c r="F4" t="n">
         <v>324.0818916275529</v>
@@ -533,10 +533,10 @@
         <v>198353</v>
       </c>
       <c r="D5" t="n">
-        <v>15435.9469384059</v>
+        <v>108.2205481879358</v>
       </c>
       <c r="E5" t="n">
-        <v>263.8392639160156</v>
+        <v>237.3375549316406</v>
       </c>
       <c r="F5" t="n">
         <v>327.6820786174144</v>
@@ -596,16 +596,16 @@
         <v>79342</v>
       </c>
       <c r="C2" t="n">
-        <v>58.40373147366022</v>
+        <v>43.81991749885466</v>
       </c>
       <c r="D2" t="n">
-        <v>147.0802153966373</v>
+        <v>149.9828960701772</v>
       </c>
       <c r="E2" t="n">
-        <v>0.03772276978145245</v>
+        <v>0.03888230697486829</v>
       </c>
       <c r="F2" t="n">
-        <v>11669638.45</v>
+        <v>11899942.94</v>
       </c>
     </row>
     <row r="3">
@@ -616,16 +616,16 @@
         <v>79341</v>
       </c>
       <c r="C3" t="n">
-        <v>102.8116503264635</v>
+        <v>82.34749243634782</v>
       </c>
       <c r="D3" t="n">
-        <v>182.9908050062389</v>
+        <v>191.6828139297463</v>
       </c>
       <c r="E3" t="n">
-        <v>0.05860778160093773</v>
+        <v>0.06061178961696979</v>
       </c>
       <c r="F3" t="n">
-        <v>14518673.46</v>
+        <v>15208306.14</v>
       </c>
     </row>
     <row r="4">
@@ -636,16 +636,16 @@
         <v>79341</v>
       </c>
       <c r="C4" t="n">
-        <v>134.2694555210882</v>
+        <v>111.2007897285026</v>
       </c>
       <c r="D4" t="n">
-        <v>218.1427303663932</v>
+        <v>221.0309456649148</v>
       </c>
       <c r="E4" t="n">
-        <v>0.07111077500913777</v>
+        <v>0.07365674745717851</v>
       </c>
       <c r="F4" t="n">
-        <v>17307662.37</v>
+        <v>17536816.26</v>
       </c>
     </row>
     <row r="5">
@@ -656,16 +656,16 @@
         <v>79342</v>
       </c>
       <c r="C5" t="n">
-        <v>163.6998624271563</v>
+        <v>138.8675810037497</v>
       </c>
       <c r="D5" t="n">
-        <v>247.5893202843387</v>
+        <v>253.9437884096695</v>
       </c>
       <c r="E5" t="n">
-        <v>0.08401603186206549</v>
+        <v>0.08295732398981624</v>
       </c>
       <c r="F5" t="n">
-        <v>19644231.85</v>
+        <v>20148408.06</v>
       </c>
     </row>
     <row r="6">
@@ -673,19 +673,19 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>79342</v>
+        <v>79341</v>
       </c>
       <c r="C6" t="n">
-        <v>194.1685512377621</v>
+        <v>167.8114526986917</v>
       </c>
       <c r="D6" t="n">
-        <v>270.6427334828969</v>
+        <v>274.1305083122219</v>
       </c>
       <c r="E6" t="n">
-        <v>0.09338055506541303</v>
+        <v>0.09502022913752033</v>
       </c>
       <c r="F6" t="n">
-        <v>21473335.76</v>
+        <v>21749788.66</v>
       </c>
     </row>
     <row r="7">
@@ -693,19 +693,19 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>79340</v>
+        <v>79341</v>
       </c>
       <c r="C7" t="n">
-        <v>228.1939974743262</v>
+        <v>201.0770840334902</v>
       </c>
       <c r="D7" t="n">
-        <v>286.9531454499622</v>
+        <v>298.8393617423527</v>
       </c>
       <c r="E7" t="n">
-        <v>0.10302495588606</v>
+        <v>0.1025825235376413</v>
       </c>
       <c r="F7" t="n">
-        <v>22766862.56</v>
+        <v>23710213.8</v>
       </c>
     </row>
     <row r="8">
@@ -716,16 +716,16 @@
         <v>79342</v>
       </c>
       <c r="C8" t="n">
-        <v>270.0215209670924</v>
+        <v>241.814537454128</v>
       </c>
       <c r="D8" t="n">
-        <v>317.7203346273096</v>
+        <v>325.4925619470142</v>
       </c>
       <c r="E8" t="n">
-        <v>0.1130170653626074</v>
+        <v>0.1142900355423357</v>
       </c>
       <c r="F8" t="n">
-        <v>25208566.79</v>
+        <v>25825230.85</v>
       </c>
     </row>
     <row r="9">
@@ -736,16 +736,16 @@
         <v>79341</v>
       </c>
       <c r="C9" t="n">
-        <v>327.1964119197822</v>
+        <v>297.4642725088327</v>
       </c>
       <c r="D9" t="n">
-        <v>393.9007123681325</v>
+        <v>382.1370283964155</v>
       </c>
       <c r="E9" t="n">
-        <v>0.1308402969460934</v>
+        <v>0.1312184116660995</v>
       </c>
       <c r="F9" t="n">
-        <v>31252476.42</v>
+        <v>30319133.97</v>
       </c>
     </row>
     <row r="10">
@@ -756,16 +756,16 @@
         <v>79341</v>
       </c>
       <c r="C10" t="n">
-        <v>420.5471689774251</v>
+        <v>388.9464276537918</v>
       </c>
       <c r="D10" t="n">
-        <v>470.0572461904942</v>
+        <v>466.4243048360873</v>
       </c>
       <c r="E10" t="n">
-        <v>0.1557958684664927</v>
+        <v>0.1536658222104587</v>
       </c>
       <c r="F10" t="n">
-        <v>37294811.97</v>
+        <v>37006570.77</v>
       </c>
     </row>
     <row r="11">
@@ -776,16 +776,16 @@
         <v>79342</v>
       </c>
       <c r="C11" t="n">
-        <v>746.7109228970107</v>
+        <v>705.0365606797766</v>
       </c>
       <c r="D11" t="n">
-        <v>755.8582023392403</v>
+        <v>727.2711763000681</v>
       </c>
       <c r="E11" t="n">
-        <v>0.228895162713317</v>
+        <v>0.2235260013611958</v>
       </c>
       <c r="F11" t="n">
-        <v>59971301.49</v>
+        <v>57703149.67</v>
       </c>
     </row>
   </sheetData>
@@ -822,92 +822,92 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>exposure</t>
+          <t>ncb_years</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>337757.6796875</v>
+        <v>59937.1923828125</v>
       </c>
       <c r="C2" t="n">
-        <v>23.01294141425816</v>
+        <v>9.338115980978216</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>telematics_opt_in</t>
+          <t>cover_type</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>99048.8125</v>
+        <v>31421.158203125</v>
       </c>
       <c r="C3" t="n">
-        <v>6.748638613704625</v>
+        <v>4.895364762557437</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ncb_years</t>
+          <t>make_model</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>85442.42578125</v>
+        <v>30597.5771484375</v>
       </c>
       <c r="C4" t="n">
-        <v>5.821574628932935</v>
+        <v>4.767052188967259</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>make_model</t>
+          <t>written_premium</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>67591.6103515625</v>
+        <v>29799.1181640625</v>
       </c>
       <c r="C5" t="n">
-        <v>4.605318731923535</v>
+        <v>4.642653592607815</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>transmission</t>
+          <t>voluntary_excess</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>47191.2001953125</v>
+        <v>25491.6220703125</v>
       </c>
       <c r="C6" t="n">
-        <v>3.21534754255788</v>
+        <v>3.971552786715169</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>voluntary_excess</t>
+          <t>prior_claims_5y</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>44025.0146484375</v>
+        <v>25101.7783203125</v>
       </c>
       <c r="C7" t="n">
-        <v>2.999621159772683</v>
+        <v>3.910815771729405</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>cover_type</t>
+          <t>payment_method</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>41310.9521484375</v>
+        <v>24532.89013671875</v>
       </c>
       <c r="C8" t="n">
-        <v>2.814699942393044</v>
+        <v>3.822183928504632</v>
       </c>
     </row>
     <row r="9">
@@ -917,114 +917,114 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>38200.8046875</v>
+        <v>22288.72412109375</v>
       </c>
       <c r="C9" t="n">
-        <v>2.602791685045706</v>
+        <v>3.472546554757953</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>annual_mileage</t>
+          <t>driver_age</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>37367.39453125</v>
+        <v>21183.99755859375</v>
       </c>
       <c r="C10" t="n">
-        <v>2.546007723486122</v>
+        <v>3.300431973514228</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>written_premium</t>
+          <t>missed_payments_12m</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>37051.724609375</v>
+        <v>21065.2333984375</v>
       </c>
       <c r="C11" t="n">
-        <v>2.524499719804092</v>
+        <v>3.281928712720175</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>prior_claims_5y</t>
+          <t>new_business</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>34366.466796875</v>
+        <v>20394.63134765625</v>
       </c>
       <c r="C12" t="n">
-        <v>2.341541094619267</v>
+        <v>3.177450016299404</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>channel</t>
+          <t>annual_mileage</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>32866.58203125</v>
+        <v>19799.07666015625</v>
       </c>
       <c r="C13" t="n">
-        <v>2.239347236965454</v>
+        <v>3.084663575630472</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>missed_payments_12m</t>
+          <t>channel</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>29609.12060546875</v>
+        <v>17198.9697265625</v>
       </c>
       <c r="C14" t="n">
-        <v>2.017401820298489</v>
+        <v>2.679571192360838</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>region</t>
+          <t>named_young_driver</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>28761.30859375</v>
+        <v>15975.20385742188</v>
       </c>
       <c r="C15" t="n">
-        <v>1.959636595910283</v>
+        <v>2.488910482953389</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>driver_age</t>
+          <t>urban_density</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>27931.20751953125</v>
+        <v>15366.2001953125</v>
       </c>
       <c r="C16" t="n">
-        <v>1.903078096910103</v>
+        <v>2.394028714162888</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>payment_method</t>
+          <t>vehicle_use</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>27858.8916015625</v>
+        <v>14765.56225585938</v>
       </c>
       <c r="C17" t="n">
-        <v>1.898150889969692</v>
+        <v>2.300450311201233</v>
       </c>
     </row>
     <row r="18">
@@ -1034,75 +1034,75 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>25876.23974609375</v>
+        <v>14097.78857421875</v>
       </c>
       <c r="C18" t="n">
-        <v>1.763063951200492</v>
+        <v>2.196412270040113</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>seats</t>
+          <t>licence_points</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>25854.78442382812</v>
+        <v>12940.36938476562</v>
       </c>
       <c r="C19" t="n">
-        <v>1.761602104130783</v>
+        <v>2.016088264192579</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>new_business</t>
+          <t>exposure</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>25620.2783203125</v>
+        <v>12821.34814453125</v>
       </c>
       <c r="C20" t="n">
-        <v>1.745624154416999</v>
+        <v>1.997544950745232</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>urban_density</t>
+          <t>marketing_segment</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>25296.5615234375</v>
+        <v>12783.70971679688</v>
       </c>
       <c r="C21" t="n">
-        <v>1.723567881149762</v>
+        <v>1.991680945616656</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>marketing_segment</t>
+          <t>telematics_score</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>25249.5517578125</v>
+        <v>12359.1806640625</v>
       </c>
       <c r="C22" t="n">
-        <v>1.720364895555986</v>
+        <v>1.925540017519643</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>body_type</t>
+          <t>region</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>22230.08471679688</v>
+        <v>12289.82763671875</v>
       </c>
       <c r="C23" t="n">
-        <v>1.514635100806488</v>
+        <v>1.914734929940105</v>
       </c>
     </row>
     <row r="24">
@@ -1112,88 +1112,88 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>22080.962890625</v>
+        <v>12114.04809570312</v>
       </c>
       <c r="C24" t="n">
-        <v>1.504474763808509</v>
+        <v>1.887348766594261</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>vehicle_age</t>
+          <t>credit_band</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>21560.3564453125</v>
+        <v>11836.96044921875</v>
       </c>
       <c r="C25" t="n">
-        <v>1.469003518160012</v>
+        <v>1.844178967060751</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>days_quote_to_inception</t>
+          <t>vehicle_age</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>21132.08911132812</v>
+        <v>11785.35815429688</v>
       </c>
       <c r="C26" t="n">
-        <v>1.439823749173732</v>
+        <v>1.836139414393895</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>named_young_driver</t>
+          <t>telematics_opt_in</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>21003.017578125</v>
+        <v>10578.86450195312</v>
       </c>
       <c r="C27" t="n">
-        <v>1.431029528315157</v>
+        <v>1.648169687951876</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>credit_band</t>
+          <t>Year</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>20796.6845703125</v>
+        <v>10156.73266601562</v>
       </c>
       <c r="C28" t="n">
-        <v>1.416971137622131</v>
+        <v>1.582402242288572</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>vehicle_use</t>
+          <t>body_type</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>20768.54833984375</v>
+        <v>10109.5517578125</v>
       </c>
       <c r="C29" t="n">
-        <v>1.415054090394679</v>
+        <v>1.575051534399641</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>telematics_score</t>
+          <t>seats</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>19051.962890625</v>
+        <v>10084.13500976562</v>
       </c>
       <c r="C30" t="n">
-        <v>1.298095445925104</v>
+        <v>1.571091646862615</v>
       </c>
     </row>
     <row r="31">
@@ -1203,127 +1203,127 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>18519.04370117188</v>
+        <v>9796.626220703125</v>
       </c>
       <c r="C31" t="n">
-        <v>1.26178527794679</v>
+        <v>1.526298250457446</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>licence_points</t>
+          <t>branch_id</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>18111.216796875</v>
+        <v>9730.883544921875</v>
       </c>
       <c r="C32" t="n">
-        <v>1.233998206859536</v>
+        <v>1.516055649712583</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>branch_id</t>
+          <t>overnight_parking</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>17990.23828125</v>
+        <v>9584.86376953125</v>
       </c>
       <c r="C33" t="n">
-        <v>1.225755399486399</v>
+        <v>1.493306008898493</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>hail_days</t>
+          <t>renewal_count</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>17271.58959960938</v>
+        <v>9493.26953125</v>
       </c>
       <c r="C34" t="n">
-        <v>1.176790650488445</v>
+        <v>1.479035777240045</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>engine_size_cc</t>
+          <t>hail_days</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>17233.77734375</v>
+        <v>9491.8095703125</v>
       </c>
       <c r="C35" t="n">
-        <v>1.174214332372932</v>
+        <v>1.478808317727511</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>renewal_count</t>
+          <t>days_quote_to_inception</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>16677.9794921875</v>
+        <v>9394.8310546875</v>
       </c>
       <c r="C36" t="n">
-        <v>1.136345338815147</v>
+        <v>1.463699224515647</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>driver_assist</t>
+          <t>transmission</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>15359.33984375</v>
+        <v>9307.105224609375</v>
       </c>
       <c r="C37" t="n">
-        <v>1.046500521654848</v>
+        <v>1.450031684492</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>overnight_parking</t>
+          <t>marital_status</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>13383.57788085938</v>
+        <v>9032.489501953125</v>
       </c>
       <c r="C38" t="n">
-        <v>0.9118830220835884</v>
+        <v>1.40724700662478</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>marital_status</t>
+          <t>engine_size_cc</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>13371.4072265625</v>
+        <v>8684.60888671875</v>
       </c>
       <c r="C39" t="n">
-        <v>0.9110537809703551</v>
+        <v>1.353047779009237</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Year</t>
+          <t>driver_assist</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>6865.338989257812</v>
+        <v>8462.002807617188</v>
       </c>
       <c r="C40" t="n">
-        <v>0.467766252110061</v>
+        <v>1.318366118055807</v>
       </c>
     </row>
   </sheetData>

</xml_diff>